<commit_message>
Fix parallel execution and update ignore list
</commit_message>
<xml_diff>
--- a/Strategy.xlsx
+++ b/Strategy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dilekozturk/git/esg-with-feature-expressions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69330C6-4F6A-7B41-B158-1256AE781634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB7AC8F-B1A0-7C47-81AA-51055AAEB6AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="15080" xr2:uid="{44512E93-00E1-D749-8DD0-3ACD2105363E}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="15060" xr2:uid="{44512E93-00E1-D749-8DD0-3ACD2105363E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -80,9 +80,6 @@
     <t>Random Walk Fault Detection</t>
   </si>
   <si>
-    <t>Fault Detection Rate</t>
-  </si>
-  <si>
     <t>Impact of Fault Types on Detection Latency</t>
   </si>
   <si>
@@ -179,6 +176,9 @@
   </si>
   <si>
     <t>RQ4(Optimal Coverage): At what coverage level L do the gains in fault detection effectiveness no longer justify the additional test generation and execution cost?</t>
+  </si>
+  <si>
+    <t>Mutation Score</t>
   </si>
 </sst>
 </file>
@@ -613,6 +613,78 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -634,33 +706,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -671,51 +716,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1076,57 +1076,57 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="8"/>
+      <c r="A2" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="32"/>
     </row>
     <row r="3" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="12"/>
+      <c r="A3" s="33"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="36"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="24" t="s">
+      <c r="C4" s="38"/>
+      <c r="D4" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="25"/>
-      <c r="F4" s="22" t="s">
+      <c r="E4" s="40"/>
+      <c r="F4" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="23"/>
-      <c r="H4" s="24" t="s">
+      <c r="G4" s="38"/>
+      <c r="H4" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="23"/>
-      <c r="J4" s="24" t="s">
+      <c r="I4" s="38"/>
+      <c r="J4" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="25"/>
+      <c r="K4" s="40"/>
     </row>
     <row r="5" spans="1:13" ht="17" x14ac:dyDescent="0.2">
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1135,10 +1135,10 @@
       <c r="D5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="27" t="s">
+      <c r="E5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="26" t="s">
+      <c r="F5" s="6" t="s">
         <v>9</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -1153,15 +1153,15 @@
       <c r="J5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="27" t="s">
+      <c r="K5" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="51" x14ac:dyDescent="0.2">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="2">
@@ -1170,10 +1170,10 @@
       <c r="D6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="7">
         <v>11</v>
       </c>
-      <c r="F6" s="26" t="s">
+      <c r="F6" s="6" t="s">
         <v>7</v>
       </c>
       <c r="G6" s="2">
@@ -1188,21 +1188,21 @@
       <c r="J6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K6" s="27">
+      <c r="K6" s="7">
         <v>11</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="26" t="s">
+      <c r="A7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C7" s="2">
@@ -1211,10 +1211,10 @@
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="7">
         <v>11</v>
       </c>
-      <c r="F7" s="26" t="s">
+      <c r="F7" s="6" t="s">
         <v>8</v>
       </c>
       <c r="G7" s="2">
@@ -1229,282 +1229,282 @@
       <c r="J7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K7" s="27">
+      <c r="K7" s="7">
         <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
-      <c r="K8" s="31"/>
-      <c r="L8" s="32"/>
-      <c r="M8" s="32"/>
+      <c r="B8" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="29"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B9" s="33"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="33"/>
-      <c r="L9" s="32"/>
-      <c r="M9" s="32"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+    </row>
+    <row r="12" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="28"/>
+      <c r="D12" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="28"/>
+    </row>
+    <row r="13" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="7">
+        <v>11</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="7">
+        <v>11</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="7">
+        <v>3</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="26"/>
+      <c r="D16" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="26"/>
+    </row>
+    <row r="17" spans="1:19" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="11">
+        <v>47.97</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+    </row>
+    <row r="18" spans="1:19" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="11">
+        <v>426.67200000000003</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+    </row>
+    <row r="19" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+      <c r="A19" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A22" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="13"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
-    </row>
-    <row r="12" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="34" t="s">
-        <v>1</v>
-      </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="34" t="s">
-        <v>3</v>
-      </c>
-      <c r="E12" s="35"/>
-    </row>
-    <row r="13" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="27" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="27" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="B14" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="27">
+      <c r="B22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="16"/>
+      <c r="N22" s="16"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="16"/>
+      <c r="Q22" s="16"/>
+      <c r="R22" s="16"/>
+      <c r="S22" s="16"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A23" s="16"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="16"/>
+      <c r="N23" s="16"/>
+      <c r="O23" s="16"/>
+      <c r="P23" s="16"/>
+      <c r="Q23" s="16"/>
+      <c r="R23" s="16"/>
+      <c r="S23" s="16"/>
+    </row>
+    <row r="24" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="27">
-        <v>11</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="27">
-        <v>3</v>
-      </c>
-      <c r="D15" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" s="27">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="29" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="31"/>
-      <c r="D16" s="29" t="s">
-        <v>18</v>
-      </c>
-      <c r="E16" s="31"/>
-    </row>
-    <row r="17" spans="1:19" ht="17" x14ac:dyDescent="0.2">
-      <c r="A17" s="36" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" s="36">
-        <v>47.97</v>
-      </c>
-      <c r="C17" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="33"/>
-      <c r="I17" s="33"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="33"/>
-      <c r="L17" s="32"/>
-      <c r="M17" s="32"/>
-    </row>
-    <row r="18" spans="1:19" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="36">
-        <v>426.67200000000003</v>
-      </c>
-      <c r="C18" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="33"/>
-      <c r="I18" s="33"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="33"/>
-      <c r="L18" s="32"/>
-      <c r="M18" s="32"/>
-    </row>
-    <row r="19" spans="1:19" ht="68" x14ac:dyDescent="0.2">
-      <c r="A19" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="36" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="D19" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="33"/>
-      <c r="I19" s="33"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="33"/>
-      <c r="L19" s="32"/>
-      <c r="M19" s="32"/>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A22" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13"/>
-      <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="13"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="13"/>
-      <c r="O22" s="13"/>
-      <c r="P22" s="13"/>
-      <c r="Q22" s="13"/>
-      <c r="R22" s="13"/>
-      <c r="S22" s="13"/>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
-      <c r="P23" s="13"/>
-      <c r="Q23" s="13"/>
-      <c r="R23" s="13"/>
-      <c r="S23" s="13"/>
-    </row>
-    <row r="24" spans="1:19" s="37" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="15"/>
-      <c r="L24" s="15"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="14" t="s">
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="I24" s="23"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
+      <c r="M24" s="24"/>
+      <c r="N24" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="O24" s="15"/>
-      <c r="P24" s="15"/>
-      <c r="Q24" s="15"/>
-      <c r="R24" s="15"/>
-      <c r="S24" s="16"/>
-    </row>
-    <row r="25" spans="1:19" ht="17" x14ac:dyDescent="0.2">
+      <c r="O24" s="23"/>
+      <c r="P24" s="23"/>
+      <c r="Q24" s="23"/>
+      <c r="R24" s="23"/>
+      <c r="S24" s="24"/>
+    </row>
+    <row r="25" spans="1:19" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="17" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>9</v>
@@ -1513,16 +1513,16 @@
         <v>10</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G25" s="27" t="s">
+      <c r="G25" s="7" t="s">
         <v>10</v>
       </c>
       <c r="H25" s="17" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>9</v>
@@ -1531,16 +1531,16 @@
         <v>10</v>
       </c>
       <c r="K25" s="19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="L25" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="M25" s="27" t="s">
+      <c r="M25" s="7" t="s">
         <v>10</v>
       </c>
       <c r="N25" s="17" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="O25" s="2" t="s">
         <v>9</v>
@@ -1549,17 +1549,17 @@
         <v>10</v>
       </c>
       <c r="Q25" s="19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R25" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="S25" s="27" t="s">
+      <c r="S25" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:19" ht="17" x14ac:dyDescent="0.2">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B26" s="17"/>
@@ -1573,7 +1573,7 @@
       <c r="F26" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G26" s="27">
+      <c r="G26" s="7">
         <v>1</v>
       </c>
       <c r="H26" s="17"/>
@@ -1587,7 +1587,7 @@
       <c r="L26" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="M26" s="27">
+      <c r="M26" s="7">
         <v>1</v>
       </c>
       <c r="N26" s="17"/>
@@ -1601,31 +1601,31 @@
       <c r="R26" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="S26" s="27">
+      <c r="S26" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:19" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B27" s="18"/>
       <c r="C27" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D27" s="3">
         <v>1</v>
       </c>
       <c r="E27" s="21"/>
       <c r="F27" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G27" s="3">
         <v>1</v>
       </c>
       <c r="H27" s="18"/>
       <c r="I27" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J27" s="3">
         <v>1</v>
@@ -1634,7 +1634,7 @@
       <c r="L27" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M27" s="38">
+      <c r="M27" s="13">
         <v>1</v>
       </c>
       <c r="N27" s="18"/>
@@ -1648,71 +1648,71 @@
       <c r="R27" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="S27" s="38">
+      <c r="S27" s="13">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A31" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="13"/>
-      <c r="J31" s="13"/>
-      <c r="K31" s="13"/>
+      <c r="A31" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" s="16"/>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="16"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A32" s="13"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
-      <c r="J32" s="13"/>
-      <c r="K32" s="13"/>
+      <c r="A32" s="16"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="16"/>
+      <c r="I32" s="16"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="16"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A35" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B35" s="13"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
-      <c r="J35" s="13"/>
-      <c r="K35" s="13"/>
+      <c r="A35" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" s="16"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="16"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="16"/>
+      <c r="K35" s="16"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A36" s="13"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="13"/>
-      <c r="J36" s="13"/>
-      <c r="K36" s="13"/>
+      <c r="A36" s="16"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="16"/>
+      <c r="K36" s="16"/>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B37" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="C37" s="40"/>
+      <c r="B37" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C37" s="15"/>
     </row>
     <row r="38" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="B38" s="2" t="s">
@@ -1746,6 +1746,24 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A2:K3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="F8:K8"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A10:K11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="N24:S24"/>
+    <mergeCell ref="N25:N27"/>
+    <mergeCell ref="Q25:Q27"/>
+    <mergeCell ref="A22:S23"/>
+    <mergeCell ref="A31:K32"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="A35:K36"/>
     <mergeCell ref="B25:B27"/>
@@ -1754,24 +1772,6 @@
     <mergeCell ref="H24:M24"/>
     <mergeCell ref="H25:H27"/>
     <mergeCell ref="K25:K27"/>
-    <mergeCell ref="N24:S24"/>
-    <mergeCell ref="N25:N27"/>
-    <mergeCell ref="Q25:Q27"/>
-    <mergeCell ref="A22:S23"/>
-    <mergeCell ref="A31:K32"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="A10:K11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A2:K3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="F8:K8"/>
-    <mergeCell ref="F4:G4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1787,12 +1787,12 @@
   <sheetData>
     <row r="4" spans="1:1" ht="409.6" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="60" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1807,17 +1807,17 @@
   <sheetData>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1835,7 +1835,7 @@
   <sheetData>
     <row r="3" spans="1:1" ht="272" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>